<commit_message>
LCSC part number added
</commit_message>
<xml_diff>
--- a/Strommessplatine/Project Outputs for Strommessplatine/Rev01/BOM/BOM_Strommessplatine_Default_Rev01.xlsx
+++ b/Strommessplatine/Project Outputs for Strommessplatine/Rev01/BOM/BOM_Strommessplatine_Default_Rev01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhan\Documents\uz_per_external_current_sensing\Strommessplatine\Project Outputs for Strommessplatine\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B3DBE2A-14D2-4711-82EA-107091E427D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{51E03C9F-9E07-49AC-9957-2BB78271534A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1448" windowWidth="16200" windowHeight="9315" xr2:uid="{09813E2A-7630-4BCE-9C02-7CC4FDD79DB8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FEC93DA8-5942-4A42-B7E6-83154AD3A106}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_Strommessplatine_Default_Re" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="137">
   <si>
     <t>Name</t>
   </si>
@@ -62,33 +62,48 @@
     <t>CAPC1608X07N</t>
   </si>
   <si>
+    <t>C7046262</t>
+  </si>
+  <si>
     <t>7.5nF</t>
   </si>
   <si>
     <t>C2</t>
   </si>
   <si>
+    <t>C2391158</t>
+  </si>
+  <si>
     <t>10µF</t>
   </si>
   <si>
-    <t>C3, C4, C8, C9, C14, C56, C60, C62</t>
+    <t>C3, C4, C8, C9, C56, C60, C62</t>
   </si>
   <si>
     <t>C_1206</t>
   </si>
   <si>
+    <t>C96600</t>
+  </si>
+  <si>
     <t>100nF</t>
   </si>
   <si>
-    <t>C5, C7, C10, C15, C57, C61</t>
-  </si>
-  <si>
-    <t>0.027µF</t>
+    <t>C5, C7, C10, C57, C61</t>
+  </si>
+  <si>
+    <t>C14663</t>
+  </si>
+  <si>
+    <t>27nF</t>
   </si>
   <si>
     <t>C6</t>
   </si>
   <si>
+    <t>C162433</t>
+  </si>
+  <si>
     <t>1 µF</t>
   </si>
   <si>
@@ -98,28 +113,46 @@
     <t>C0603</t>
   </si>
   <si>
+    <t>C2189093</t>
+  </si>
+  <si>
+    <t>C14</t>
+  </si>
+  <si>
+    <t>C15</t>
+  </si>
+  <si>
+    <t>tbd</t>
+  </si>
+  <si>
+    <t>C16A, C16B, C16C, C16D, C18A, C18B, C18C, C18D, C20A, C20B, C20C, C20D</t>
+  </si>
+  <si>
+    <t>0.1 µF</t>
+  </si>
+  <si>
+    <t>C17A, C17B, C17C, C17D, C24A, C24B, C24C, C24D, C29A, C29B, C29C, C29D</t>
+  </si>
+  <si>
+    <t>47uF</t>
+  </si>
+  <si>
+    <t>C19</t>
+  </si>
+  <si>
+    <t>WCAP-ASLI_5x5.5</t>
+  </si>
+  <si>
+    <t>C5534035</t>
+  </si>
+  <si>
     <t>22 pF</t>
   </si>
   <si>
-    <t>C16A, C16B, C16C, C16D, C18A, C18B, C18C, C18D, C20A, C20B, C20C, C20D, C21A, C21B, C21C, C21D, C27A, C27B, C27C, C27D</t>
-  </si>
-  <si>
-    <t>0.1 µF</t>
-  </si>
-  <si>
-    <t>C17A, C17B, C17C, C17D, C24A, C24B, C24C, C24D, C29A, C29B, C29C, C29D</t>
-  </si>
-  <si>
-    <t>C14663</t>
-  </si>
-  <si>
-    <t>47uF</t>
-  </si>
-  <si>
-    <t>C19</t>
-  </si>
-  <si>
-    <t>WCAP-ASLI_5x5.5</t>
+    <t>C21A, C21B, C21C, C21D, C27A, C27B, C27C, C27D</t>
+  </si>
+  <si>
+    <t>C2169678</t>
   </si>
   <si>
     <t>2.2 nF</t>
@@ -128,12 +161,18 @@
     <t>C22A, C22B, C22C, C22D</t>
   </si>
   <si>
+    <t>C597200</t>
+  </si>
+  <si>
     <t>100 pF</t>
   </si>
   <si>
     <t>C23A, C23B, C23C, C23D, C28A, C28B, C28C, C28D</t>
   </si>
   <si>
+    <t>C6107920</t>
+  </si>
+  <si>
     <t>BYS12-90</t>
   </si>
   <si>
@@ -143,6 +182,9 @@
     <t>DIOM4227X23N</t>
   </si>
   <si>
+    <t>C3758831</t>
+  </si>
+  <si>
     <t>150060BS75000</t>
   </si>
   <si>
@@ -152,16 +194,25 @@
     <t>WL-SMCW_0603</t>
   </si>
   <si>
+    <t>C5197644</t>
+  </si>
+  <si>
     <t>150060GS75000</t>
   </si>
   <si>
     <t>D3</t>
   </si>
   <si>
+    <t>C5252984</t>
+  </si>
+  <si>
     <t>150060RS75000</t>
   </si>
   <si>
-    <t>D4</t>
+    <t>D4, D5</t>
+  </si>
+  <si>
+    <t>C3030991</t>
   </si>
   <si>
     <t>68001-202HLF</t>
@@ -185,6 +236,9 @@
     <t>J3</t>
   </si>
   <si>
+    <t>C5157943</t>
+  </si>
+  <si>
     <t>600Ω</t>
   </si>
   <si>
@@ -194,6 +248,9 @@
     <t>WE-CBF_0805_High Current</t>
   </si>
   <si>
+    <t>C2661857</t>
+  </si>
+  <si>
     <t>150uH</t>
   </si>
   <si>
@@ -203,6 +260,9 @@
     <t>SMT_inductor_1050_Performance</t>
   </si>
   <si>
+    <t>C2045822</t>
+  </si>
+  <si>
     <t>Mounting Hole</t>
   </si>
   <si>
@@ -212,6 +272,18 @@
     <t>MH_3.4</t>
   </si>
   <si>
+    <t>499R</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R0603</t>
+  </si>
+  <si>
+    <t>C103675</t>
+  </si>
+  <si>
     <t>162k</t>
   </si>
   <si>
@@ -227,18 +299,27 @@
     <t>R8</t>
   </si>
   <si>
+    <t>C4243723</t>
+  </si>
+  <si>
     <t>1.62k</t>
   </si>
   <si>
     <t>R9</t>
   </si>
   <si>
+    <t>C2077223</t>
+  </si>
+  <si>
     <t>133k</t>
   </si>
   <si>
     <t>R10</t>
   </si>
   <si>
+    <t>C2084976</t>
+  </si>
+  <si>
     <t>1.02k</t>
   </si>
   <si>
@@ -251,12 +332,18 @@
     <t>R11A, R11B, R11C, R11D, R16A, R16B, R16C, R16D</t>
   </si>
   <si>
+    <t>C1861697</t>
+  </si>
+  <si>
     <t>1k 0.1%</t>
   </si>
   <si>
     <t>R12A, R12B, R12C, R12D, R14A, R14B, R14C, R14D</t>
   </si>
   <si>
+    <t>C22396727</t>
+  </si>
+  <si>
     <t>49R9</t>
   </si>
   <si>
@@ -272,24 +359,36 @@
     <t>R21</t>
   </si>
   <si>
+    <t>C19946998</t>
+  </si>
+  <si>
     <t>10k</t>
   </si>
   <si>
     <t>R24</t>
   </si>
   <si>
+    <t>C840630</t>
+  </si>
+  <si>
     <t>6.04k</t>
   </si>
   <si>
     <t>R28, R56</t>
   </si>
   <si>
+    <t>C4178162</t>
+  </si>
+  <si>
     <t>24.9k</t>
   </si>
   <si>
     <t>R55</t>
   </si>
   <si>
+    <t>C2077039</t>
+  </si>
+  <si>
     <t>LM5007</t>
   </si>
   <si>
@@ -299,6 +398,9 @@
     <t>TSOP65P490X110-8N</t>
   </si>
   <si>
+    <t>C23920</t>
+  </si>
+  <si>
     <t>REF35250QDBVR</t>
   </si>
   <si>
@@ -326,6 +428,9 @@
     <t>ADA4940-1ARZ-R7</t>
   </si>
   <si>
+    <t>C459899</t>
+  </si>
+  <si>
     <t>TPS7A49</t>
   </si>
   <si>
@@ -333,6 +438,9 @@
   </si>
   <si>
     <t>DGN0008D_N</t>
+  </si>
+  <si>
+    <t>C16430</t>
   </si>
   <si>
     <t>Pin Spring Probe Connector</t>
@@ -348,7 +456,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -737,17 +845,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD29C0B-9207-4D83-9D7D-1332383FCC77}">
-  <dimension ref="A1:D40"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B55397-F513-496C-941E-7617EB5FB40B}">
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="16.875" customWidth="1"/>
-    <col min="2" max="2" width="15.625" customWidth="1"/>
-    <col min="3" max="3" width="21.5" customWidth="1"/>
-    <col min="4" max="4" width="14.625" customWidth="1"/>
+    <col min="1" max="1" width="17.9296875" customWidth="1"/>
+    <col min="2" max="2" width="16.59765625" customWidth="1"/>
+    <col min="3" max="3" width="22.86328125" customWidth="1"/>
+    <col min="4" max="4" width="15.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1">
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -761,7 +869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -771,472 +879,584 @@
       <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="D5" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4">
+        <v>33</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4">
+        <v>46</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4">
+        <v>50</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4">
+        <v>50</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="1:4">
+        <v>58</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D21" s="1"/>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="1"/>
-    </row>
-    <row r="23" spans="1:4">
+        <v>63</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="1"/>
-    </row>
-    <row r="24" spans="1:4">
+        <v>68</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="1:4">
+        <v>72</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="D25" s="1"/>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="1:4">
+        <v>79</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="D27" s="1"/>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D28" s="1"/>
-    </row>
-    <row r="29" spans="1:4">
+        <v>83</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D29" s="1"/>
-    </row>
-    <row r="30" spans="1:4">
+        <v>83</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>18</v>
+        <v>83</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="D31" s="1"/>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="1"/>
-    </row>
-    <row r="33" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D33" s="1"/>
-    </row>
-    <row r="34" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" s="1"/>
-    </row>
-    <row r="35" spans="1:4">
+        <v>23</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" s="1"/>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="D35" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D37" s="1"/>
-    </row>
-    <row r="38" spans="1:4">
+        <v>83</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D38" s="1"/>
-    </row>
-    <row r="39" spans="1:4">
+        <v>83</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D39" s="1"/>
-    </row>
-    <row r="40" spans="1:4">
+        <v>118</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>100</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A41" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D41" s="1"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A43" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A44" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
switching node compacter renamed 2V5 bypass capacitors displaced in phases
</commit_message>
<xml_diff>
--- a/Strommessplatine/Project Outputs for Strommessplatine/Rev01/BOM/BOM_Strommessplatine_Default_Rev01.xlsx
+++ b/Strommessplatine/Project Outputs for Strommessplatine/Rev01/BOM/BOM_Strommessplatine_Default_Rev01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhan\Documents\uz_per_external_current_sensing\Strommessplatine\Project Outputs for Strommessplatine\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51E03C9F-9E07-49AC-9957-2BB78271534A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EABDFE1-6954-4635-910D-752BCEF7440C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FEC93DA8-5942-4A42-B7E6-83154AD3A106}"/>
   </bookViews>
@@ -850,7 +850,7 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.9296875" customWidth="1"/>
-    <col min="2" max="2" width="16.59765625" customWidth="1"/>
+    <col min="2" max="2" width="63.9296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.86328125" customWidth="1"/>
     <col min="4" max="4" width="15.53125" customWidth="1"/>
   </cols>

</xml_diff>